<commit_message>
feat: integrate model explainability backend and populate comprehensive financial evaluation artifacts and paper visualizations.
</commit_message>
<xml_diff>
--- a/result.xlsx
+++ b/result.xlsx
@@ -474,16 +474,16 @@
         <v>0.9251305861868834</v>
       </c>
       <c r="E2" t="n">
-        <v>0.9294386923273236</v>
+        <v>0.9209800523754244</v>
       </c>
       <c r="F2" t="n">
         <v>0.9251305861868834</v>
       </c>
       <c r="G2" t="n">
-        <v>0.9267141416007784</v>
+        <v>0.9222594171823576</v>
       </c>
       <c r="H2" t="n">
-        <v>0.9803353706554868</v>
+        <v>0.9805595628619184</v>
       </c>
     </row>
     <row r="3">
@@ -499,19 +499,19 @@
       </c>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="n">
-        <v>0.9239698200812536</v>
+        <v>0.9193267556587348</v>
       </c>
       <c r="E3" t="n">
-        <v>0.9244634057572086</v>
+        <v>0.9175586571360664</v>
       </c>
       <c r="F3" t="n">
-        <v>0.9239698200812536</v>
+        <v>0.9193267556587348</v>
       </c>
       <c r="G3" t="n">
-        <v>0.9242007139355536</v>
+        <v>0.9178421751225684</v>
       </c>
       <c r="H3" t="n">
-        <v>0.958443027777124</v>
+        <v>0.9533908544040796</v>
       </c>
     </row>
     <row r="4">
@@ -527,19 +527,19 @@
       </c>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="n">
-        <v>0.9251305861868834</v>
+        <v>0.922228670922809</v>
       </c>
       <c r="E4" t="n">
-        <v>0.9257928678184248</v>
+        <v>0.9205064124293486</v>
       </c>
       <c r="F4" t="n">
-        <v>0.9251305861868834</v>
+        <v>0.922228670922809</v>
       </c>
       <c r="G4" t="n">
-        <v>0.9254392236408068</v>
+        <v>0.9204071591208632</v>
       </c>
       <c r="H4" t="n">
-        <v>0.947930578940096</v>
+        <v>0.9533034661195652</v>
       </c>
     </row>
     <row r="5">
@@ -555,19 +555,19 @@
       </c>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="n">
-        <v>0.9239698200812536</v>
+        <v>0.9135229251305862</v>
       </c>
       <c r="E5" t="n">
-        <v>0.9244181521169244</v>
+        <v>0.9079060861632452</v>
       </c>
       <c r="F5" t="n">
-        <v>0.9239698200812536</v>
+        <v>0.9135229251305862</v>
       </c>
       <c r="G5" t="n">
-        <v>0.9241654197927832</v>
+        <v>0.9073087290061844</v>
       </c>
       <c r="H5" t="n">
-        <v>0.952838588053554</v>
+        <v>0.9484985916018092</v>
       </c>
     </row>
     <row r="6">
@@ -583,19 +583,19 @@
       </c>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="n">
-        <v>0.9199071387115496</v>
+        <v>0.9204875217643644</v>
       </c>
       <c r="E6" t="n">
-        <v>0.9184111867906072</v>
+        <v>0.9193771148303872</v>
       </c>
       <c r="F6" t="n">
-        <v>0.9199071387115496</v>
+        <v>0.9204875217643644</v>
       </c>
       <c r="G6" t="n">
-        <v>0.9185275533977512</v>
+        <v>0.9194961953210752</v>
       </c>
       <c r="H6" t="n">
-        <v>0.964094215513572</v>
+        <v>0.9646821175270764</v>
       </c>
     </row>
     <row r="7">
@@ -611,19 +611,19 @@
       </c>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="n">
-        <v>0.91874637260592</v>
+        <v>0.9199071387115496</v>
       </c>
       <c r="E7" t="n">
-        <v>0.9178029276156654</v>
+        <v>0.9188479563463277</v>
       </c>
       <c r="F7" t="n">
-        <v>0.91874637260592</v>
+        <v>0.9199071387115496</v>
       </c>
       <c r="G7" t="n">
-        <v>0.9180203288186412</v>
+        <v>0.9190185928764512</v>
       </c>
       <c r="H7" t="n">
-        <v>0.9654027336187068</v>
+        <v>0.9656378713856985</v>
       </c>
     </row>
     <row r="8">
@@ -643,19 +643,19 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.92397</v>
+        <v>0.925131</v>
       </c>
       <c r="E8" t="n">
-        <v>0.9249039999999999</v>
+        <v>0.9218</v>
       </c>
       <c r="F8" t="n">
-        <v>0.92397</v>
+        <v>0.9251</v>
       </c>
       <c r="G8" t="n">
-        <v>0.924399</v>
+        <v>0.9221</v>
       </c>
       <c r="H8" t="n">
-        <v>0.981999</v>
+        <v>0.9733039999999999</v>
       </c>
     </row>
     <row r="9">
@@ -675,19 +675,19 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.92397</v>
+        <v>0.923389</v>
       </c>
       <c r="E9" t="n">
-        <v>0.923573</v>
+        <v>0.922</v>
       </c>
       <c r="F9" t="n">
-        <v>0.92397</v>
+        <v>0.9234</v>
       </c>
       <c r="G9" t="n">
-        <v>0.92366</v>
+        <v>0.9222</v>
       </c>
       <c r="H9" t="n">
-        <v>0.965804</v>
+        <v>0.962025</v>
       </c>
     </row>
     <row r="10">
@@ -707,19 +707,19 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.9257</v>
+        <v>0.921648</v>
       </c>
       <c r="E10" t="n">
-        <v>0.9266</v>
+        <v>0.9175</v>
       </c>
       <c r="F10" t="n">
-        <v>0.9257</v>
+        <v>0.9216</v>
       </c>
       <c r="G10" t="n">
-        <v>0.9261</v>
+        <v>0.9182</v>
       </c>
       <c r="H10" t="n">
-        <v>0.982</v>
+        <v>0.972421</v>
       </c>
     </row>
     <row r="11">
@@ -739,19 +739,19 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.925711</v>
+        <v>0.922809</v>
       </c>
       <c r="E11" t="n">
-        <v>0.926427</v>
+        <v>0.9209000000000001</v>
       </c>
       <c r="F11" t="n">
-        <v>0.925711</v>
+        <v>0.9228</v>
       </c>
       <c r="G11" t="n">
-        <v>0.9260429999999999</v>
+        <v>0.9204</v>
       </c>
       <c r="H11" t="n">
-        <v>0.981501</v>
+        <v>0.97268</v>
       </c>
     </row>
     <row r="12">
@@ -774,16 +774,16 @@
         <v>0.92397</v>
       </c>
       <c r="E12" t="n">
-        <v>0.923573</v>
+        <v>0.9226</v>
       </c>
       <c r="F12" t="n">
-        <v>0.92397</v>
+        <v>0.924</v>
       </c>
       <c r="G12" t="n">
-        <v>0.92366</v>
+        <v>0.9227</v>
       </c>
       <c r="H12" t="n">
-        <v>0.965804</v>
+        <v>0.9610300000000001</v>
       </c>
     </row>
     <row r="13">
@@ -803,19 +803,19 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.923389</v>
+        <v>0.92455</v>
       </c>
       <c r="E13" t="n">
-        <v>0.923924</v>
+        <v>0.9233</v>
       </c>
       <c r="F13" t="n">
-        <v>0.923389</v>
+        <v>0.9246</v>
       </c>
       <c r="G13" t="n">
-        <v>0.923645</v>
+        <v>0.9231</v>
       </c>
       <c r="H13" t="n">
-        <v>0.981301</v>
+        <v>0.971125</v>
       </c>
     </row>
     <row r="14">
@@ -831,19 +831,19 @@
       </c>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="n">
-        <v>0.905398</v>
+        <v>0.9233894370284388</v>
       </c>
       <c r="E14" t="n">
-        <v>0.904745</v>
+        <v>0.923484968301122</v>
       </c>
       <c r="F14" t="n">
-        <v>0.905398</v>
+        <v>0.9233894370284388</v>
       </c>
       <c r="G14" t="n">
-        <v>0.903659</v>
+        <v>0.923424283112033</v>
       </c>
       <c r="H14" t="n">
-        <v>0.950667</v>
+        <v>0.930629442132104</v>
       </c>
     </row>
     <row r="15">
@@ -863,19 +863,19 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0.919327</v>
+        <v>0.929774</v>
       </c>
       <c r="E15" t="n">
-        <v>0.919466</v>
+        <v>0.926706</v>
       </c>
       <c r="F15" t="n">
-        <v>0.919327</v>
+        <v>0.929774</v>
       </c>
       <c r="G15" t="n">
-        <v>0.915169</v>
+        <v>0.925974</v>
       </c>
       <c r="H15" t="n">
-        <v>0.954297</v>
+        <v>0.948986</v>
       </c>
     </row>
   </sheetData>

</xml_diff>